<commit_message>
Adding export/import and supply
</commit_message>
<xml_diff>
--- a/VT_EE_UPS_V01.xlsx
+++ b/VT_EE_UPS_V01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67818AE0-98CB-49AB-9A13-5891C522BC49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C06CE32-0FDD-4B0C-B379-F906750CAE57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="901" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" tabRatio="901" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EB1" sheetId="133" r:id="rId1"/>
@@ -1883,6 +1883,8 @@
     <author>Gary Goldstein</author>
     <author>Amit Kanudia</author>
     <author>Maurizio Gargiulo</author>
+    <author>tc={74C5EBC3-3855-49CC-8D22-3D22C507954E}</author>
+    <author>tc={E7A732B9-0C2E-4BF2-B78D-5BF686EADA9E}</author>
   </authors>
   <commentList>
     <comment ref="I3" authorId="0" shapeId="0" xr:uid="{6E5AAF16-2CE6-41AB-BA3C-4DE6B7722EEA}">
@@ -2653,6 +2655,22 @@
           </rPr>
           <t xml:space="preserve"> (Heating Plant)</t>
         </r>
+      </text>
+    </comment>
+    <comment ref="W10" authorId="3" shapeId="0" xr:uid="{74C5EBC3-3855-49CC-8D22-3D22C507954E}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    https://news.err.ee/1609986120/vkg-overtakes-enefit-as-estonia-s-largest-oil-shale-miner</t>
+      </text>
+    </comment>
+    <comment ref="Y10" authorId="4" shapeId="0" xr:uid="{E7A732B9-0C2E-4BF2-B78D-5BF686EADA9E}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Approx</t>
       </text>
     </comment>
   </commentList>
@@ -7359,7 +7377,7 @@
     <author>Maurizio Gargiulo</author>
   </authors>
   <commentList>
-    <comment ref="H3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0800-000001000000}">
+    <comment ref="J3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0800-000001000000}">
       <text>
         <r>
           <rPr>
@@ -7473,7 +7491,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M3" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0800-000002000000}">
+    <comment ref="O3" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0800-000002000000}">
       <text>
         <r>
           <rPr>
@@ -7499,7 +7517,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N3" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0800-000003000000}">
+    <comment ref="P3" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0800-000003000000}">
       <text>
         <r>
           <rPr>
@@ -7572,7 +7590,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O3" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0800-000004000000}">
+    <comment ref="Q3" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0800-000004000000}">
       <text>
         <r>
           <rPr>
@@ -7625,7 +7643,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P3" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0800-000005000000}">
+    <comment ref="R3" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0800-000005000000}">
       <text>
         <r>
           <rPr>
@@ -7705,7 +7723,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N12" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0800-000007000000}">
+    <comment ref="P12" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0800-000007000000}">
       <text>
         <r>
           <rPr>
@@ -7798,7 +7816,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O12" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0800-000008000000}">
+    <comment ref="Q12" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0800-000008000000}">
       <text>
         <r>
           <rPr>
@@ -7823,7 +7841,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P12" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0800-000009000000}">
+    <comment ref="R12" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0800-000009000000}">
       <text>
         <r>
           <rPr>
@@ -7886,7 +7904,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H13" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0800-00000A000000}">
+    <comment ref="J13" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0800-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -8134,7 +8152,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="741" uniqueCount="172">
   <si>
     <t>CommName</t>
   </si>
@@ -8588,17 +8606,81 @@
   <si>
     <t>Oil shale</t>
   </si>
+  <si>
+    <t>ktoe2PJ</t>
+  </si>
+  <si>
+    <t>total mined (t)</t>
+  </si>
+  <si>
+    <t>Energy density of oil shale (MJ/kg)</t>
+  </si>
+  <si>
+    <t>Production (PJ)</t>
+  </si>
+  <si>
+    <t>Cost (€/t)</t>
+  </si>
+  <si>
+    <t>Energy density of oil shale (tons/PJ)</t>
+  </si>
+  <si>
+    <t>Cost (M€/PJ)</t>
+  </si>
+  <si>
+    <t>TWh</t>
+  </si>
+  <si>
+    <t>Cap2ACT</t>
+  </si>
+  <si>
+    <t>Import of Electricity from Finland</t>
+  </si>
+  <si>
+    <t>IMPELCFIN</t>
+  </si>
+  <si>
+    <t>IMPELCLV</t>
+  </si>
+  <si>
+    <t>Import of Electricity from Latvia</t>
+  </si>
+  <si>
+    <t>EXPELCFIN</t>
+  </si>
+  <si>
+    <t>Export of Electricity to Finland</t>
+  </si>
+  <si>
+    <t>EXPELCLV</t>
+  </si>
+  <si>
+    <t>Export of Electricity to Latvia</t>
+  </si>
+  <si>
+    <t>GW</t>
+  </si>
+  <si>
+    <t>NCAP_PASTI</t>
+  </si>
+  <si>
+    <t>FLO_COST</t>
+  </si>
+  <si>
+    <t>NCAP_AF</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="General_)"/>
     <numFmt numFmtId="165" formatCode="\Te\x\t"/>
+    <numFmt numFmtId="171" formatCode="0.000"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -8761,6 +8843,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="16">
@@ -9125,7 +9213,7 @@
     <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -9315,6 +9403,12 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="171" fontId="4" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="22">
     <cellStyle name="20% - Accent5" xfId="1" builtinId="46"/>
@@ -9441,15 +9535,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>809625</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>2486057</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>2247932</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -9464,7 +9558,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7200900" y="6076950"/>
+          <a:off x="6838950" y="7362825"/>
           <a:ext cx="4514882" cy="1047750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9549,13 +9643,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>428625</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>57150</xdr:rowOff>
@@ -9938,13 +10032,13 @@
     <xdr:from>
       <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>2299252</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -10304,13 +10398,13 @@
     <xdr:from>
       <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -11131,6 +11225,12 @@
 </externalLink>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Kristopher Raik" id="{618EE9E7-879B-4C97-88A2-981A8E483D41}" userId="S::krraik@taltech.ee::b956339b-354b-46f9-8dd3-3584d8dbf762" providerId="AD"/>
+</personList>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -11477,6 +11577,23 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="W10" dT="2026-09-21T06:53:58.90" personId="{618EE9E7-879B-4C97-88A2-981A8E483D41}" id="{74C5EBC3-3855-49CC-8D22-3D22C507954E}">
+    <text>https://news.err.ee/1609986120/vkg-overtakes-enefit-as-estonia-s-largest-oil-shale-miner</text>
+    <extLst>
+      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
+        <xltc2:checksum>4246205987</xltc2:checksum>
+        <xltc2:hyperlink startIndex="0" length="88" url="https://news.err.ee/1609986120/vkg-overtakes-enefit-as-estonia-s-largest-oil-shale-miner"/>
+      </x:ext>
+    </extLst>
+  </threadedComment>
+  <threadedComment ref="Y10" dT="2026-09-21T06:56:12.74" personId="{618EE9E7-879B-4C97-88A2-981A8E483D41}" id="{E7A732B9-0C2E-4BF2-B78D-5BF686EADA9E}">
+    <text>Approx</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
@@ -12393,28 +12510,28 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="B1:S22"/>
+  <dimension ref="B1:U22"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" customWidth="1"/>
-    <col min="7" max="7" width="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.140625" customWidth="1"/>
-    <col min="10" max="10" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="37.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11" customWidth="1"/>
-    <col min="14" max="14" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" customWidth="1"/>
+    <col min="6" max="8" width="13.7109375" customWidth="1"/>
+    <col min="9" max="9" width="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.140625" customWidth="1"/>
+    <col min="12" max="12" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="37.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11" customWidth="1"/>
+    <col min="16" max="16" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:21" ht="30" x14ac:dyDescent="0.25">
       <c r="B1" s="24" t="s">
         <v>66</v>
       </c>
@@ -12430,8 +12547,10 @@
       <c r="F1" s="24" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="2" spans="2:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+    </row>
+    <row r="2" spans="2:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B2" s="9" t="s">
         <v>112</v>
       </c>
@@ -12443,130 +12562,131 @@
         <f>'EB1'!U$3</f>
         <v>Electricity</v>
       </c>
-      <c r="E2" s="9" t="str">
-        <f>'EB1'!$Z$2</f>
-        <v>PJ</v>
+      <c r="E2" s="9" t="s">
+        <v>158</v>
       </c>
       <c r="F2" s="9" t="str">
         <f>'EB1'!Y2</f>
         <v>M€2025</v>
       </c>
-      <c r="H2" s="91" t="s">
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="J2" s="91" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="91"/>
-      <c r="J2" s="92"/>
-      <c r="K2" s="92"/>
+      <c r="K2" s="91"/>
       <c r="L2" s="92"/>
       <c r="M2" s="92"/>
       <c r="N2" s="92"/>
       <c r="O2" s="92"/>
       <c r="P2" s="92"/>
-    </row>
-    <row r="3" spans="2:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="Q2" s="92"/>
+      <c r="R2" s="92"/>
+    </row>
+    <row r="3" spans="2:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
-      <c r="H3" s="93" t="s">
+      <c r="J3" s="93" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="94" t="s">
+      <c r="K3" s="94" t="s">
         <v>30</v>
       </c>
-      <c r="J3" s="93" t="s">
+      <c r="L3" s="93" t="s">
         <v>0</v>
       </c>
-      <c r="K3" s="93" t="s">
+      <c r="M3" s="93" t="s">
         <v>3</v>
       </c>
-      <c r="L3" s="93" t="s">
+      <c r="N3" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="M3" s="93" t="s">
+      <c r="O3" s="93" t="s">
         <v>8</v>
       </c>
-      <c r="N3" s="93" t="s">
+      <c r="P3" s="93" t="s">
         <v>9</v>
       </c>
-      <c r="O3" s="93" t="s">
+      <c r="Q3" s="93" t="s">
         <v>10</v>
       </c>
-      <c r="P3" s="93" t="s">
+      <c r="R3" s="93" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="2:19" ht="24" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:21" ht="24" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
-      <c r="H4" s="95" t="s">
+      <c r="J4" s="95" t="s">
         <v>37</v>
       </c>
-      <c r="I4" s="95" t="s">
+      <c r="K4" s="95" t="s">
         <v>31</v>
       </c>
-      <c r="J4" s="95" t="s">
+      <c r="L4" s="95" t="s">
         <v>26</v>
       </c>
-      <c r="K4" s="95" t="s">
+      <c r="M4" s="95" t="s">
         <v>27</v>
       </c>
-      <c r="L4" s="95" t="s">
+      <c r="N4" s="95" t="s">
         <v>4</v>
       </c>
-      <c r="M4" s="95" t="s">
+      <c r="O4" s="95" t="s">
         <v>40</v>
       </c>
-      <c r="N4" s="95" t="s">
+      <c r="P4" s="95" t="s">
         <v>41</v>
       </c>
-      <c r="O4" s="95" t="s">
+      <c r="Q4" s="95" t="s">
         <v>28</v>
       </c>
-      <c r="P4" s="95" t="s">
+      <c r="R4" s="95" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="2:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
-      <c r="H5" s="1"/>
       <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
-    </row>
-    <row r="6" spans="2:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="Q5" s="1"/>
+      <c r="R5" s="1"/>
+    </row>
+    <row r="6" spans="2:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
-      <c r="H6" s="1"/>
       <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
-    </row>
-    <row r="11" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="Q6" s="1"/>
+      <c r="R6" s="1"/>
+    </row>
+    <row r="11" spans="2:21" x14ac:dyDescent="0.2">
       <c r="D11" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E11" s="4"/>
-      <c r="H11" s="91" t="s">
+      <c r="J11" s="91" t="s">
         <v>15</v>
       </c>
-      <c r="I11" s="91"/>
-      <c r="J11" s="96"/>
-      <c r="K11" s="96"/>
+      <c r="K11" s="91"/>
       <c r="L11" s="96"/>
       <c r="M11" s="96"/>
       <c r="N11" s="96"/>
       <c r="O11" s="96"/>
       <c r="P11" s="96"/>
-    </row>
-    <row r="12" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="Q11" s="96"/>
+      <c r="R11" s="96"/>
+    </row>
+    <row r="12" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B12" s="3" t="s">
         <v>1</v>
       </c>
@@ -12577,40 +12697,46 @@
         <v>6</v>
       </c>
       <c r="E12" s="53" t="s">
-        <v>35</v>
+        <v>170</v>
       </c>
       <c r="F12" s="53" t="s">
-        <v>72</v>
-      </c>
-      <c r="H12" s="93" t="s">
+        <v>169</v>
+      </c>
+      <c r="G12" s="99" t="s">
+        <v>159</v>
+      </c>
+      <c r="H12" s="99" t="s">
+        <v>171</v>
+      </c>
+      <c r="J12" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="I12" s="94" t="s">
+      <c r="K12" s="94" t="s">
         <v>30</v>
       </c>
-      <c r="J12" s="93" t="s">
+      <c r="L12" s="93" t="s">
         <v>1</v>
       </c>
-      <c r="K12" s="93" t="s">
+      <c r="M12" s="93" t="s">
         <v>2</v>
       </c>
-      <c r="L12" s="93" t="s">
+      <c r="N12" s="93" t="s">
         <v>16</v>
       </c>
-      <c r="M12" s="93" t="s">
+      <c r="O12" s="93" t="s">
         <v>17</v>
       </c>
-      <c r="N12" s="93" t="s">
+      <c r="P12" s="93" t="s">
         <v>18</v>
       </c>
-      <c r="O12" s="93" t="s">
+      <c r="Q12" s="93" t="s">
         <v>19</v>
       </c>
-      <c r="P12" s="93" t="s">
+      <c r="R12" s="93" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="2:19" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:21" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B13" s="12" t="s">
         <v>39</v>
       </c>
@@ -12626,35 +12752,37 @@
       <c r="F13" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="H13" s="95" t="s">
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+      <c r="J13" s="95" t="s">
         <v>38</v>
       </c>
-      <c r="I13" s="95" t="s">
+      <c r="K13" s="95" t="s">
         <v>31</v>
       </c>
-      <c r="J13" s="95" t="s">
+      <c r="L13" s="95" t="s">
         <v>21</v>
       </c>
-      <c r="K13" s="95" t="s">
+      <c r="M13" s="95" t="s">
         <v>22</v>
       </c>
-      <c r="L13" s="95" t="s">
+      <c r="N13" s="95" t="s">
         <v>23</v>
       </c>
-      <c r="M13" s="95" t="s">
+      <c r="O13" s="95" t="s">
         <v>24</v>
       </c>
-      <c r="N13" s="95" t="s">
+      <c r="P13" s="95" t="s">
         <v>43</v>
       </c>
-      <c r="O13" s="95" t="s">
+      <c r="Q13" s="95" t="s">
         <v>42</v>
       </c>
-      <c r="P13" s="95" t="s">
+      <c r="R13" s="95" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="2:19" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:21" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B14" s="12" t="s">
         <v>77</v>
       </c>
@@ -12662,28 +12790,30 @@
       <c r="D14" s="11"/>
       <c r="E14" s="11" t="str">
         <f>$F$2&amp;"/"&amp;$E$2</f>
-        <v>M€2025/PJ</v>
-      </c>
-      <c r="F14" s="11" t="str">
-        <f>$E$2</f>
-        <v>PJ</v>
-      </c>
-      <c r="H14" s="95" t="s">
+        <v>M€2025/TWh</v>
+      </c>
+      <c r="F14" s="97" t="str">
+        <f>O15</f>
+        <v>GW</v>
+      </c>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="J14" s="95" t="s">
         <v>73</v>
       </c>
-      <c r="I14" s="95"/>
-      <c r="J14" s="95"/>
       <c r="K14" s="95"/>
       <c r="L14" s="95"/>
       <c r="M14" s="95"/>
       <c r="N14" s="95"/>
       <c r="O14" s="95"/>
       <c r="P14" s="95"/>
-    </row>
-    <row r="15" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="Q14" s="95"/>
+      <c r="R14" s="95"/>
+    </row>
+    <row r="15" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B15" s="1" t="str">
-        <f>J15</f>
-        <v>IMPELC1</v>
+        <f>L15</f>
+        <v>IMPELCFIN</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1" t="str">
@@ -12691,86 +12821,168 @@
         <v>ELC</v>
       </c>
       <c r="E15" s="49">
-        <f>Pri_GAS!F12*1.3</f>
-        <v>5.3819999999999997</v>
-      </c>
-      <c r="F15" s="44">
-        <f>'EB1'!U6</f>
-        <v>583.76</v>
-      </c>
-      <c r="H15" s="96" t="str">
+        <v>80.39</v>
+      </c>
+      <c r="F15" s="101">
+        <v>1.016</v>
+      </c>
+      <c r="G15" s="100">
+        <v>8.76</v>
+      </c>
+      <c r="H15" s="100">
+        <v>0.9</v>
+      </c>
+      <c r="J15" s="96" t="str">
         <f>'EB1'!$B$6</f>
         <v>IMP</v>
       </c>
-      <c r="I15" s="96"/>
-      <c r="J15" s="96" t="str">
-        <f>$H$15&amp;C2&amp;1</f>
-        <v>IMPELC1</v>
-      </c>
-      <c r="K15" s="98" t="str">
-        <f>"Import of "&amp;D2&amp; " Step "&amp;RIGHT(J15,1)</f>
-        <v>Import of Electricity Step 1</v>
-      </c>
-      <c r="L15" s="96" t="str">
+      <c r="K15" s="96"/>
+      <c r="L15" s="96" t="s">
+        <v>161</v>
+      </c>
+      <c r="M15" s="98" t="s">
+        <v>160</v>
+      </c>
+      <c r="N15" s="96" t="str">
         <f>$E$2</f>
-        <v>PJ</v>
-      </c>
-      <c r="M15" s="96"/>
-      <c r="N15" s="92" t="s">
+        <v>TWh</v>
+      </c>
+      <c r="O15" s="96" t="s">
+        <v>168</v>
+      </c>
+      <c r="P15" s="92" t="s">
         <v>92</v>
       </c>
-      <c r="O15" s="96"/>
-      <c r="P15" s="96"/>
-    </row>
-    <row r="16" spans="2:19" x14ac:dyDescent="0.2">
+      <c r="Q15" s="96"/>
+      <c r="R15" s="96"/>
+    </row>
+    <row r="16" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="str">
-        <f>J16</f>
-        <v>EXPELC1</v>
-      </c>
-      <c r="C16" s="1" t="str">
+        <f>L16</f>
+        <v>IMPELCLV</v>
+      </c>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1" t="str">
         <f>C2</f>
         <v>ELC</v>
       </c>
-      <c r="D16" s="1"/>
       <c r="E16" s="49">
-        <v>6</v>
-      </c>
-      <c r="F16" s="44">
-        <f>-'EB1'!U$7</f>
-        <v>563.40200000000004</v>
-      </c>
-      <c r="H16" s="96" t="str">
+        <v>85.31</v>
+      </c>
+      <c r="F16" s="101">
+        <v>1.149</v>
+      </c>
+      <c r="G16" s="100">
+        <v>8.76</v>
+      </c>
+      <c r="H16" s="100"/>
+      <c r="J16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L16" t="s">
+        <v>162</v>
+      </c>
+      <c r="M16" t="s">
+        <v>163</v>
+      </c>
+      <c r="N16" s="96" t="str">
+        <f t="shared" ref="N16:N18" si="0">$E$2</f>
+        <v>TWh</v>
+      </c>
+      <c r="O16" s="96" t="s">
+        <v>168</v>
+      </c>
+      <c r="P16" s="92" t="s">
+        <v>92</v>
+      </c>
+      <c r="U16" s="1"/>
+    </row>
+    <row r="17" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B17" s="1" t="str">
+        <f>L17</f>
+        <v>EXPELCFIN</v>
+      </c>
+      <c r="C17" t="str">
+        <f>C2</f>
+        <v>ELC</v>
+      </c>
+      <c r="E17">
+        <v>40.49</v>
+      </c>
+      <c r="F17" s="102">
+        <v>1.016</v>
+      </c>
+      <c r="H17" s="51"/>
+      <c r="J17" s="96" t="str">
         <f>'EB1'!B7</f>
         <v>EXP</v>
       </c>
-      <c r="I16" s="96"/>
-      <c r="J16" s="96" t="str">
-        <f>$H$16&amp;C2&amp;1</f>
-        <v>EXPELC1</v>
-      </c>
-      <c r="K16" s="98" t="str">
-        <f>"Export of "&amp;D2&amp; " Step "&amp;RIGHT(J16,1)</f>
-        <v>Export of Electricity Step 1</v>
-      </c>
-      <c r="L16" s="96" t="str">
-        <f>$E$2</f>
-        <v>PJ</v>
-      </c>
-      <c r="M16" s="96"/>
-      <c r="N16" s="92" t="s">
+      <c r="K17" s="96"/>
+      <c r="L17" s="96" t="s">
+        <v>164</v>
+      </c>
+      <c r="M17" s="98" t="s">
+        <v>165</v>
+      </c>
+      <c r="N17" s="96" t="str">
+        <f t="shared" si="0"/>
+        <v>TWh</v>
+      </c>
+      <c r="O17" s="96" t="s">
+        <v>168</v>
+      </c>
+      <c r="P17" s="92" t="s">
         <v>92</v>
       </c>
-      <c r="O16" s="96"/>
-      <c r="P16" s="96"/>
-      <c r="S16" s="1"/>
-    </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="Q17" s="96"/>
+      <c r="R17" s="96"/>
+    </row>
+    <row r="18" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B18" s="1" t="str">
+        <f>L18</f>
+        <v>EXPELCLV</v>
+      </c>
+      <c r="C18" t="str">
+        <f>C2</f>
+        <v>ELC</v>
+      </c>
+      <c r="E18">
+        <v>85.31</v>
+      </c>
+      <c r="F18" s="102">
+        <v>0.85</v>
+      </c>
+      <c r="H18" s="51"/>
+      <c r="J18" t="s">
+        <v>62</v>
+      </c>
+      <c r="L18" t="s">
+        <v>166</v>
+      </c>
+      <c r="M18" t="s">
+        <v>167</v>
+      </c>
+      <c r="N18" s="96" t="str">
+        <f t="shared" si="0"/>
+        <v>TWh</v>
+      </c>
+      <c r="O18" s="96" t="s">
+        <v>168</v>
+      </c>
+      <c r="P18" s="92" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="19" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="H19" s="51"/>
+    </row>
+    <row r="21" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B21" s="38"/>
       <c r="C21" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B22" s="46"/>
       <c r="C22" s="1" t="s">
         <v>115</v>
@@ -13107,10 +13319,7 @@
         <f>-SUM('EB1'!F13)/SUM('EB1'!G13:M13)</f>
         <v>1.0128203720739584</v>
       </c>
-      <c r="G12" s="45">
-        <f>SUM('EB1'!G13:M13)</f>
-        <v>15667.368999999999</v>
-      </c>
+      <c r="G12" s="45"/>
       <c r="H12" s="5"/>
       <c r="J12" s="92" t="s">
         <v>87</v>
@@ -13417,7 +13626,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="B1:R26"/>
+  <dimension ref="B1:R23"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
@@ -13711,35 +13920,28 @@
     <row r="11" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="str">
         <f>K11</f>
-        <v>MINCOA1</v>
+        <v>IMPCOA1</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1" t="str">
         <f>$K$5</f>
         <v>COA</v>
       </c>
-      <c r="E11" s="48">
-        <v>80000</v>
-      </c>
-      <c r="F11" s="50">
-        <v>2</v>
-      </c>
-      <c r="G11" s="44">
-        <f>'EB1'!$D$5*'EB1'!D21</f>
-        <v>3947.949525</v>
-      </c>
-      <c r="I11" s="92" t="str">
-        <f>'EB1'!$B$5</f>
-        <v>MIN</v>
+      <c r="E11" s="1"/>
+      <c r="F11" s="50"/>
+      <c r="G11" s="5"/>
+      <c r="I11" s="96" t="str">
+        <f>'EB1'!$B$6</f>
+        <v>IMP</v>
       </c>
       <c r="J11" s="96"/>
       <c r="K11" s="96" t="str">
         <f>$I$11&amp;$C$2&amp;1</f>
-        <v>MINCOA1</v>
+        <v>IMPCOA1</v>
       </c>
       <c r="L11" s="98" t="str">
-        <f>"Domestic Supply of "&amp;$D$2&amp; " Step "&amp;RIGHT(K11,1)</f>
-        <v>Domestic Supply of Solid Fuels Step 1</v>
+        <f>"Import of "&amp;$D$2&amp; " Step "&amp;RIGHT(K11,1)</f>
+        <v>Import of Solid Fuels Step 1</v>
       </c>
       <c r="M11" s="96" t="str">
         <f>$E$2</f>
@@ -13756,32 +13958,27 @@
     <row r="12" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B12" s="1" t="str">
         <f>K12</f>
-        <v>MINCOA2</v>
-      </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1" t="str">
+        <v>EXPCOA1</v>
+      </c>
+      <c r="C12" s="1" t="str">
         <f>$K$5</f>
         <v>COA</v>
       </c>
-      <c r="E12" s="48">
-        <v>160000</v>
-      </c>
-      <c r="F12" s="50">
-        <v>2.5</v>
-      </c>
-      <c r="G12" s="44">
-        <f>'EB1'!$D$5*'EB1'!D22</f>
-        <v>1315.9831750000001</v>
-      </c>
-      <c r="I12" s="96"/>
+      <c r="D12" s="1"/>
+      <c r="F12" s="50"/>
+      <c r="G12" s="45"/>
+      <c r="I12" s="96" t="str">
+        <f>'EB1'!B7</f>
+        <v>EXP</v>
+      </c>
       <c r="J12" s="96"/>
       <c r="K12" s="96" t="str">
-        <f>$I$11&amp;$C$2&amp;2</f>
-        <v>MINCOA2</v>
+        <f>$I$12&amp;$C$2&amp;1</f>
+        <v>EXPCOA1</v>
       </c>
       <c r="L12" s="98" t="str">
-        <f>"Domestic Supply of "&amp;$D$2&amp; " Step "&amp;RIGHT(K12,1)</f>
-        <v>Domestic Supply of Solid Fuels Step 2</v>
+        <f>"Export of "&amp;$D$2&amp; " Step "&amp;RIGHT(K12,1)</f>
+        <v>Export of Solid Fuels Step 1</v>
       </c>
       <c r="M12" s="96" t="str">
         <f>$E$2</f>
@@ -13796,165 +13993,44 @@
       <c r="Q12" s="96"/>
     </row>
     <row r="13" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B13" s="1" t="str">
-        <f>K13</f>
-        <v>MINCOA3</v>
-      </c>
+      <c r="B13" s="1"/>
       <c r="C13" s="1"/>
-      <c r="D13" s="1" t="str">
-        <f>$K$5</f>
-        <v>COA</v>
-      </c>
-      <c r="E13" s="48">
-        <v>3000000</v>
-      </c>
-      <c r="F13" s="50">
-        <v>3</v>
-      </c>
+      <c r="E13" s="1"/>
       <c r="G13" s="10"/>
-      <c r="I13" s="96"/>
-      <c r="J13" s="96"/>
-      <c r="K13" s="96" t="str">
-        <f>$I$11&amp;$C$2&amp;3</f>
-        <v>MINCOA3</v>
-      </c>
-      <c r="L13" s="98" t="str">
-        <f>"Domestic Supply of "&amp;$D$2&amp; " Step "&amp;RIGHT(K13,1)</f>
-        <v>Domestic Supply of Solid Fuels Step 3</v>
-      </c>
-      <c r="M13" s="96" t="str">
-        <f>$E$2</f>
-        <v>PJ</v>
-      </c>
-      <c r="N13" s="96" t="str">
-        <f>$E$2&amp;"a"</f>
-        <v>PJa</v>
-      </c>
-      <c r="O13" s="96"/>
-      <c r="P13" s="96"/>
-      <c r="Q13" s="96"/>
     </row>
     <row r="14" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B14" s="1" t="str">
-        <f>K14</f>
-        <v>IMPCOA1</v>
-      </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1" t="str">
-        <f>$K$5</f>
-        <v>COA</v>
-      </c>
-      <c r="E14" s="1"/>
-      <c r="F14" s="50">
-        <v>2.75</v>
-      </c>
-      <c r="G14" s="5"/>
-      <c r="I14" s="96" t="str">
-        <f>'EB1'!$B$6</f>
-        <v>IMP</v>
-      </c>
-      <c r="J14" s="96"/>
-      <c r="K14" s="96" t="str">
-        <f>$I$14&amp;$C$2&amp;1</f>
-        <v>IMPCOA1</v>
-      </c>
-      <c r="L14" s="98" t="str">
-        <f>"Import of "&amp;$D$2&amp; " Step "&amp;RIGHT(K14,1)</f>
-        <v>Import of Solid Fuels Step 1</v>
-      </c>
-      <c r="M14" s="96" t="str">
-        <f>$E$2</f>
-        <v>PJ</v>
-      </c>
-      <c r="N14" s="96" t="str">
-        <f>$E$2&amp;"a"</f>
-        <v>PJa</v>
-      </c>
-      <c r="O14" s="96"/>
-      <c r="P14" s="96"/>
-      <c r="Q14" s="96"/>
-    </row>
-    <row r="15" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B15" s="1" t="str">
-        <f>K15</f>
-        <v>EXPCOA1</v>
-      </c>
-      <c r="C15" s="1" t="str">
-        <f>$K$5</f>
-        <v>COA</v>
-      </c>
-      <c r="D15" s="1"/>
-      <c r="F15" s="50">
-        <v>2.75</v>
-      </c>
-      <c r="G15" s="45">
-        <f>-'EB1'!D7</f>
-        <v>745.59484999999995</v>
-      </c>
-      <c r="I15" s="96" t="str">
-        <f>'EB1'!B7</f>
-        <v>EXP</v>
-      </c>
-      <c r="J15" s="96"/>
-      <c r="K15" s="96" t="str">
-        <f>$I$15&amp;$C$2&amp;1</f>
-        <v>EXPCOA1</v>
-      </c>
-      <c r="L15" s="98" t="str">
-        <f>"Export of "&amp;$D$2&amp; " Step "&amp;RIGHT(K15,1)</f>
-        <v>Export of Solid Fuels Step 1</v>
-      </c>
-      <c r="M15" s="96" t="str">
-        <f>$E$2</f>
-        <v>PJ</v>
-      </c>
-      <c r="N15" s="96" t="str">
-        <f>$E$2&amp;"a"</f>
-        <v>PJa</v>
-      </c>
-      <c r="O15" s="96"/>
-      <c r="P15" s="96"/>
-      <c r="Q15" s="96"/>
-    </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="G16" s="10"/>
-    </row>
-    <row r="17" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B17" s="1"/>
-    </row>
-    <row r="22" spans="2:18" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C22"/>
-      <c r="D22"/>
-      <c r="E22"/>
-      <c r="F22"/>
-      <c r="G22"/>
-      <c r="H22"/>
-      <c r="I22"/>
-      <c r="J22"/>
-      <c r="K22"/>
-      <c r="L22"/>
-      <c r="M22"/>
-      <c r="N22"/>
-      <c r="O22"/>
-      <c r="P22"/>
-      <c r="Q22"/>
-      <c r="R22"/>
+      <c r="B14" s="1"/>
+    </row>
+    <row r="19" spans="2:18" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="C19"/>
+      <c r="D19"/>
+      <c r="E19"/>
+      <c r="F19"/>
+      <c r="G19"/>
+      <c r="H19"/>
+      <c r="I19"/>
+      <c r="J19"/>
+      <c r="K19"/>
+      <c r="L19"/>
+      <c r="M19"/>
+      <c r="N19"/>
+      <c r="O19"/>
+      <c r="P19"/>
+      <c r="Q19"/>
+      <c r="R19"/>
+    </row>
+    <row r="20" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="R20" s="1"/>
+    </row>
+    <row r="22" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B22" s="48"/>
+      <c r="C22" s="1" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="23" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="R23" s="1"/>
-    </row>
-    <row r="25" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B25" s="48"/>
-      <c r="C25" s="1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="26" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B26" s="46"/>
-      <c r="C26" s="1" t="s">
+      <c r="B23" s="46"/>
+      <c r="C23" s="1" t="s">
         <v>115</v>
       </c>
     </row>
@@ -13969,7 +14045,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CE3D601-8357-4014-BBD5-DE38AC19BE99}">
-  <dimension ref="B1:R26"/>
+  <dimension ref="B1:Z26"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
@@ -13989,9 +14065,13 @@
     <col min="15" max="15" width="13" customWidth="1"/>
     <col min="16" max="16" width="15.140625" customWidth="1"/>
     <col min="17" max="17" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:26" ht="30" x14ac:dyDescent="0.25">
       <c r="B1" s="24" t="s">
         <v>66</v>
       </c>
@@ -14008,7 +14088,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B2" s="9"/>
       <c r="C2" s="9" t="s">
         <v>149</v>
@@ -14036,7 +14116,7 @@
       <c r="P2" s="92"/>
       <c r="Q2" s="92"/>
     </row>
-    <row r="3" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:26" x14ac:dyDescent="0.2">
       <c r="I3" s="93" t="s">
         <v>7</v>
       </c>
@@ -14065,8 +14145,13 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="2:17" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="1"/>
+    <row r="4" spans="2:26" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>151</v>
+      </c>
+      <c r="C4">
+        <v>4.1868000000000002E-2</v>
+      </c>
       <c r="I4" s="95" t="s">
         <v>37</v>
       </c>
@@ -14095,7 +14180,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:26" x14ac:dyDescent="0.2">
       <c r="I5" s="92" t="s">
         <v>65</v>
       </c>
@@ -14117,7 +14202,15 @@
       <c r="P5" s="92"/>
       <c r="Q5" s="92"/>
     </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:26" x14ac:dyDescent="0.2">
+      <c r="V6" t="s">
+        <v>153</v>
+      </c>
+      <c r="W6">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="7" spans="2:26" x14ac:dyDescent="0.2">
       <c r="D7" s="4" t="s">
         <v>13</v>
       </c>
@@ -14133,8 +14226,15 @@
       <c r="O7" s="96"/>
       <c r="P7" s="96"/>
       <c r="Q7" s="96"/>
-    </row>
-    <row r="8" spans="2:17" x14ac:dyDescent="0.2">
+      <c r="V7" t="s">
+        <v>156</v>
+      </c>
+      <c r="W7">
+        <f>1000000000/(W6*1000)</f>
+        <v>105263.15789473684</v>
+      </c>
+    </row>
+    <row r="8" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B8" s="3" t="s">
         <v>1</v>
       </c>
@@ -14181,7 +14281,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="2:17" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:26" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
         <v>39</v>
       </c>
@@ -14227,8 +14327,20 @@
       <c r="Q9" s="95" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="10" spans="2:17" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="W9" t="s">
+        <v>152</v>
+      </c>
+      <c r="X9" t="s">
+        <v>154</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>155</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="10" spans="2:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B10" s="12" t="s">
         <v>77</v>
       </c>
@@ -14257,8 +14369,25 @@
       <c r="O10" s="97"/>
       <c r="P10" s="97"/>
       <c r="Q10" s="97"/>
-    </row>
-    <row r="11" spans="2:17" x14ac:dyDescent="0.2">
+      <c r="V10">
+        <v>2025</v>
+      </c>
+      <c r="W10">
+        <v>8021108</v>
+      </c>
+      <c r="X10">
+        <f>W10*1000*W6/1000000000</f>
+        <v>76.200525999999996</v>
+      </c>
+      <c r="Y10">
+        <v>30</v>
+      </c>
+      <c r="Z10">
+        <f>W7*Y10/1000000</f>
+        <v>3.1578947368421053</v>
+      </c>
+    </row>
+    <row r="11" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="str">
         <f>K11</f>
         <v>MINSHL1</v>
@@ -14268,15 +14397,14 @@
         <f>$K$5</f>
         <v>SHL</v>
       </c>
-      <c r="E11" s="48">
-        <v>80000</v>
-      </c>
+      <c r="E11" s="48"/>
       <c r="F11" s="50">
-        <v>2</v>
+        <f>Z10</f>
+        <v>3.1578947368421053</v>
       </c>
       <c r="G11" s="44">
-        <f>'EB1'!$D$5*'EB1'!D21</f>
-        <v>3947.949525</v>
+        <f>X10</f>
+        <v>76.200525999999996</v>
       </c>
       <c r="I11" s="92" t="str">
         <f>'EB1'!$B$5</f>
@@ -14303,7 +14431,7 @@
       <c r="P11" s="96"/>
       <c r="Q11" s="96"/>
     </row>
-    <row r="12" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -14320,7 +14448,7 @@
       <c r="P12" s="96"/>
       <c r="Q12" s="96"/>
     </row>
-    <row r="13" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -14337,7 +14465,7 @@
       <c r="P13" s="96"/>
       <c r="Q13" s="96"/>
     </row>
-    <row r="14" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -14354,7 +14482,7 @@
       <c r="P14" s="96"/>
       <c r="Q14" s="96"/>
     </row>
-    <row r="15" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
@@ -14370,7 +14498,7 @@
       <c r="P15" s="96"/>
       <c r="Q15" s="96"/>
     </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="E16" s="1"/>
@@ -14722,16 +14850,11 @@
         <f>$K$5</f>
         <v>GAS</v>
       </c>
-      <c r="E11" s="43">
-        <v>15000</v>
-      </c>
+      <c r="E11" s="43"/>
       <c r="F11" s="49">
         <v>3.6</v>
       </c>
-      <c r="G11" s="45">
-        <f>'EB1'!$E$5*'EB1'!E21</f>
-        <v>1579.8994000000002</v>
-      </c>
+      <c r="G11" s="45"/>
       <c r="I11" s="92" t="str">
         <f>'EB1'!$B$5</f>
         <v>MIN</v>
@@ -14767,16 +14890,11 @@
         <f>$K$5</f>
         <v>GAS</v>
       </c>
-      <c r="E12" s="43">
-        <v>20000</v>
-      </c>
+      <c r="E12" s="43"/>
       <c r="F12" s="49">
         <v>4.1399999999999997</v>
       </c>
-      <c r="G12" s="45">
-        <f>'EB1'!$E$5*'EB1'!E22</f>
-        <v>1579.8994000000002</v>
-      </c>
+      <c r="G12" s="45"/>
       <c r="I12" s="96"/>
       <c r="J12" s="96"/>
       <c r="K12" s="96" t="str">
@@ -14809,15 +14927,11 @@
         <f>$K$5</f>
         <v>GAS</v>
       </c>
-      <c r="E13" s="49">
-        <v>0</v>
-      </c>
+      <c r="E13" s="49"/>
       <c r="F13" s="49">
         <v>5.4</v>
       </c>
-      <c r="G13" s="43">
-        <v>0</v>
-      </c>
+      <c r="G13" s="43"/>
       <c r="I13" s="96"/>
       <c r="J13" s="96"/>
       <c r="K13" s="96" t="str">
@@ -14853,10 +14967,7 @@
       <c r="F14" s="49">
         <v>4.5</v>
       </c>
-      <c r="G14" s="45">
-        <f>'EB1'!E6</f>
-        <v>5316.6916000000001</v>
-      </c>
+      <c r="G14" s="45"/>
       <c r="I14" s="96" t="str">
         <f>'EB1'!$B$6</f>
         <v>IMP</v>
@@ -14894,10 +15005,7 @@
       <c r="F15" s="49">
         <v>4.5</v>
       </c>
-      <c r="G15" s="45">
-        <f>-'EB1'!E7</f>
-        <v>1006.5324000000001</v>
-      </c>
+      <c r="G15" s="45"/>
       <c r="I15" s="96" t="str">
         <f>'EB1'!B7</f>
         <v>EXP</v>
@@ -14969,7 +15077,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="B1:W24"/>
+  <dimension ref="B1:W21"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
@@ -14991,7 +15099,7 @@
     <col min="17" max="17" width="7.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:23" ht="30" x14ac:dyDescent="0.25">
       <c r="B1" s="24" t="s">
         <v>66</v>
       </c>
@@ -15008,7 +15116,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:23" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B2" s="9"/>
       <c r="C2" s="9" t="str">
         <f>'EB1'!F2</f>
@@ -15038,7 +15146,7 @@
       <c r="P2" s="92"/>
       <c r="Q2" s="92"/>
     </row>
-    <row r="3" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:23" x14ac:dyDescent="0.2">
       <c r="I3" s="93" t="s">
         <v>7</v>
       </c>
@@ -15067,7 +15175,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="2:17" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:23" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C4" s="1"/>
       <c r="I4" s="95" t="s">
         <v>37</v>
@@ -15097,7 +15205,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:23" x14ac:dyDescent="0.2">
       <c r="I5" s="92" t="s">
         <v>65</v>
       </c>
@@ -15119,7 +15227,7 @@
       <c r="P5" s="92"/>
       <c r="Q5" s="92"/>
     </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:23" x14ac:dyDescent="0.2">
       <c r="D7" s="4" t="s">
         <v>13</v>
       </c>
@@ -15136,7 +15244,7 @@
       <c r="P7" s="96"/>
       <c r="Q7" s="96"/>
     </row>
-    <row r="8" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:23" x14ac:dyDescent="0.2">
       <c r="B8" s="3" t="s">
         <v>1</v>
       </c>
@@ -15183,7 +15291,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="2:17" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:23" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
         <v>39</v>
       </c>
@@ -15230,7 +15338,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="2:17" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B10" s="12" t="s">
         <v>77</v>
       </c>
@@ -15260,38 +15368,33 @@
       <c r="P10" s="97"/>
       <c r="Q10" s="97"/>
     </row>
-    <row r="11" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:23" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="str">
         <f>K11</f>
-        <v>MINOIL1</v>
+        <v>IMPOIL1</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1" t="str">
         <f>$K$5</f>
         <v>OIL</v>
       </c>
-      <c r="E11" s="38">
-        <v>7200</v>
-      </c>
+      <c r="E11" s="38"/>
       <c r="F11" s="49">
-        <v>6.4</v>
-      </c>
-      <c r="G11" s="45">
-        <f>'EB1'!$F$5*'EB1'!F21</f>
-        <v>2149.0016000000001</v>
-      </c>
-      <c r="I11" s="92" t="str">
-        <f>'EB1'!$B$5</f>
-        <v>MIN</v>
+        <v>8</v>
+      </c>
+      <c r="G11" s="10"/>
+      <c r="I11" s="96" t="str">
+        <f>'EB1'!$B$6</f>
+        <v>IMP</v>
       </c>
       <c r="J11" s="96"/>
       <c r="K11" s="96" t="str">
         <f>$I$11&amp;$C$2&amp;1</f>
-        <v>MINOIL1</v>
+        <v>IMPOIL1</v>
       </c>
       <c r="L11" s="98" t="str">
-        <f>"Domestic Supply of "&amp;$D$2&amp; " Step "&amp;RIGHT(K11,1)</f>
-        <v>Domestic Supply of Crude Oil Step 1</v>
+        <f>"Import of "&amp;$D$2&amp; " Step "&amp;RIGHT(K11,1)</f>
+        <v>Import of Crude Oil Step 1</v>
       </c>
       <c r="M11" s="96" t="str">
         <f>$E$2</f>
@@ -15305,35 +15408,33 @@
       <c r="P11" s="96"/>
       <c r="Q11" s="96"/>
     </row>
-    <row r="12" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:23" x14ac:dyDescent="0.2">
       <c r="B12" s="1" t="str">
         <f>K12</f>
-        <v>MINOIL2</v>
-      </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1" t="str">
+        <v>EXPOIL1</v>
+      </c>
+      <c r="C12" s="1" t="str">
         <f>$K$5</f>
         <v>OIL</v>
       </c>
-      <c r="E12" s="38">
-        <v>1800</v>
-      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="38"/>
       <c r="F12" s="49">
-        <v>7.3599999999999994</v>
-      </c>
-      <c r="G12" s="45">
-        <f>'EB1'!$F$5*'EB1'!F22</f>
-        <v>537.25040000000001</v>
-      </c>
-      <c r="I12" s="96"/>
+        <v>8</v>
+      </c>
+      <c r="G12" s="44"/>
+      <c r="I12" s="96" t="str">
+        <f>'EB1'!B7</f>
+        <v>EXP</v>
+      </c>
       <c r="J12" s="96"/>
       <c r="K12" s="96" t="str">
-        <f>$I$11&amp;$C$2&amp;2</f>
-        <v>MINOIL2</v>
+        <f>$I$12&amp;$C$2&amp;1</f>
+        <v>EXPOIL1</v>
       </c>
       <c r="L12" s="98" t="str">
-        <f>"Domestic Supply of "&amp;$D$2&amp; " Step "&amp;RIGHT(K12,1)</f>
-        <v>Domestic Supply of Crude Oil Step 2</v>
+        <f>"Export of "&amp;$D$2&amp; " Step "&amp;RIGHT(K12,1)</f>
+        <v>Export of Crude Oil Step 1</v>
       </c>
       <c r="M12" s="96" t="str">
         <f>$E$2</f>
@@ -15347,158 +15448,36 @@
       <c r="P12" s="96"/>
       <c r="Q12" s="96"/>
     </row>
-    <row r="13" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B13" s="1" t="str">
-        <f>K13</f>
-        <v>MINOIL3</v>
-      </c>
+    <row r="13" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="B13" s="1"/>
       <c r="C13" s="1"/>
-      <c r="D13" s="1" t="str">
-        <f>$K$5</f>
-        <v>OIL</v>
-      </c>
-      <c r="E13" s="38">
-        <v>1200000</v>
-      </c>
-      <c r="F13" s="49">
-        <v>9.6000000000000014</v>
-      </c>
-      <c r="G13" s="10"/>
-      <c r="I13" s="96"/>
-      <c r="J13" s="96"/>
-      <c r="K13" s="96" t="str">
-        <f>$I$11&amp;$C$2&amp;3</f>
-        <v>MINOIL3</v>
-      </c>
-      <c r="L13" s="98" t="str">
-        <f>"Domestic Supply of "&amp;$D$2&amp; " Step "&amp;RIGHT(K13,1)</f>
-        <v>Domestic Supply of Crude Oil Step 3</v>
-      </c>
-      <c r="M13" s="96" t="str">
-        <f>$E$2</f>
-        <v>PJ</v>
-      </c>
-      <c r="N13" s="96" t="str">
-        <f>$E$2&amp;"a"</f>
-        <v>PJa</v>
-      </c>
-      <c r="O13" s="96"/>
-      <c r="P13" s="96"/>
-      <c r="Q13" s="96"/>
-    </row>
-    <row r="14" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B14" s="1" t="str">
-        <f>K14</f>
-        <v>IMPOIL1</v>
-      </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1" t="str">
-        <f>$K$5</f>
-        <v>OIL</v>
-      </c>
-      <c r="E14" s="38"/>
-      <c r="F14" s="49">
-        <v>8</v>
-      </c>
-      <c r="G14" s="10"/>
-      <c r="I14" s="96" t="str">
-        <f>'EB1'!$B$6</f>
-        <v>IMP</v>
-      </c>
-      <c r="J14" s="96"/>
-      <c r="K14" s="96" t="str">
-        <f>$I$14&amp;$C$2&amp;1</f>
-        <v>IMPOIL1</v>
-      </c>
-      <c r="L14" s="98" t="str">
-        <f>"Import of "&amp;$D$2&amp; " Step "&amp;RIGHT(K14,1)</f>
-        <v>Import of Crude Oil Step 1</v>
-      </c>
-      <c r="M14" s="96" t="str">
-        <f>$E$2</f>
-        <v>PJ</v>
-      </c>
-      <c r="N14" s="96" t="str">
-        <f>$E$2&amp;"a"</f>
-        <v>PJa</v>
-      </c>
-      <c r="O14" s="96"/>
-      <c r="P14" s="96"/>
-      <c r="Q14" s="96"/>
-    </row>
-    <row r="15" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B15" s="1" t="str">
-        <f>K15</f>
-        <v>EXPOIL1</v>
-      </c>
-      <c r="C15" s="1" t="str">
-        <f>$K$5</f>
-        <v>OIL</v>
-      </c>
-      <c r="D15" s="1"/>
-      <c r="E15" s="38"/>
-      <c r="F15" s="49">
-        <v>8</v>
-      </c>
-      <c r="G15" s="44">
-        <f>-'EB1'!F7</f>
-        <v>1648.4854999999998</v>
-      </c>
-      <c r="I15" s="96" t="str">
-        <f>'EB1'!B7</f>
-        <v>EXP</v>
-      </c>
-      <c r="J15" s="96"/>
-      <c r="K15" s="96" t="str">
-        <f>$I$15&amp;$C$2&amp;1</f>
-        <v>EXPOIL1</v>
-      </c>
-      <c r="L15" s="98" t="str">
-        <f>"Export of "&amp;$D$2&amp; " Step "&amp;RIGHT(K15,1)</f>
-        <v>Export of Crude Oil Step 1</v>
-      </c>
-      <c r="M15" s="96" t="str">
-        <f>$E$2</f>
-        <v>PJ</v>
-      </c>
-      <c r="N15" s="96" t="str">
-        <f>$E$2&amp;"a"</f>
-        <v>PJa</v>
-      </c>
-      <c r="O15" s="96"/>
-      <c r="P15" s="96"/>
-      <c r="Q15" s="96"/>
-    </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="F16" s="51"/>
-    </row>
-    <row r="17" spans="2:23" x14ac:dyDescent="0.2">
-      <c r="B17" s="1"/>
-      <c r="F17" s="51"/>
-    </row>
-    <row r="18" spans="2:23" x14ac:dyDescent="0.2">
-      <c r="T18" s="1"/>
-      <c r="U18" s="1"/>
-    </row>
-    <row r="19" spans="2:23" x14ac:dyDescent="0.2">
-      <c r="S19" s="1"/>
-      <c r="V19" s="1"/>
-      <c r="W19" s="1"/>
-    </row>
-    <row r="23" spans="2:23" x14ac:dyDescent="0.2">
-      <c r="B23" s="48"/>
-      <c r="C23" s="1" t="s">
+      <c r="F13" s="51"/>
+    </row>
+    <row r="14" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="B14" s="1"/>
+      <c r="F14" s="51"/>
+    </row>
+    <row r="15" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="T15" s="1"/>
+      <c r="U15" s="1"/>
+    </row>
+    <row r="16" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="S16" s="1"/>
+      <c r="V16" s="1"/>
+      <c r="W16" s="1"/>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B20" s="48"/>
+      <c r="C20" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="24" spans="2:23" x14ac:dyDescent="0.2">
-      <c r="B24" s="46"/>
-      <c r="C24" s="1" t="s">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B21" s="46"/>
+      <c r="C21" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="H24" s="1"/>
+      <c r="H21" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17393,7 +17372,7 @@
         <v>DSL</v>
       </c>
       <c r="E17" s="49">
-        <f>Pri_OIL!$F$14*1.3</f>
+        <f>Pri_OIL!$F$11*1.3</f>
         <v>10.4</v>
       </c>
       <c r="F17" s="44"/>
@@ -17430,7 +17409,7 @@
         <v>KER</v>
       </c>
       <c r="E18" s="49">
-        <f>Pri_OIL!$F$14*1.4</f>
+        <f>Pri_OIL!$F$11*1.4</f>
         <v>11.2</v>
       </c>
       <c r="F18" s="44"/>
@@ -17465,7 +17444,7 @@
         <v>LPG</v>
       </c>
       <c r="E19" s="49">
-        <f>Pri_OIL!$F$14*1.1</f>
+        <f>Pri_OIL!$F$11*1.1</f>
         <v>8.8000000000000007</v>
       </c>
       <c r="F19" s="44"/>
@@ -17501,7 +17480,7 @@
         <v>GSL</v>
       </c>
       <c r="E20" s="49">
-        <f>Pri_OIL!$F$14*1.4</f>
+        <f>Pri_OIL!$F$11*1.4</f>
         <v>11.2</v>
       </c>
       <c r="F20" s="44"/>
@@ -17535,7 +17514,7 @@
         <v>NAP</v>
       </c>
       <c r="E21" s="49">
-        <f>Pri_OIL!$F$14*1.05</f>
+        <f>Pri_OIL!$F$11*1.05</f>
         <v>8.4</v>
       </c>
       <c r="F21" s="44"/>
@@ -17569,7 +17548,7 @@
         <v>HFO</v>
       </c>
       <c r="E22" s="49">
-        <f>Pri_OIL!$F$14*1.05</f>
+        <f>Pri_OIL!$F$11*1.05</f>
         <v>8.4</v>
       </c>
       <c r="F22" s="44"/>
@@ -17603,7 +17582,7 @@
         <v>OPP</v>
       </c>
       <c r="E23" s="49">
-        <f>Pri_OIL!$F$14*1.05</f>
+        <f>Pri_OIL!$F$11*1.05</f>
         <v>8.4</v>
       </c>
       <c r="F23" s="44"/>
@@ -17640,10 +17619,7 @@
         <f>E17*0.99</f>
         <v>10.295999999999999</v>
       </c>
-      <c r="F24" s="44">
-        <f>-'EB1'!G$7</f>
-        <v>1683.1424999999999</v>
-      </c>
+      <c r="F24" s="44"/>
       <c r="H24" s="96" t="str">
         <f>'EB1'!B7</f>
         <v>EXP</v>
@@ -17681,10 +17657,7 @@
         <f t="shared" ref="E25:E30" si="10">E18*0.99</f>
         <v>11.087999999999999</v>
       </c>
-      <c r="F25" s="44">
-        <f>-'EB1'!H$7</f>
-        <v>295.38850000000002</v>
-      </c>
+      <c r="F25" s="44"/>
       <c r="H25" s="96"/>
       <c r="I25" s="96"/>
       <c r="J25" s="96" t="str">
@@ -17719,10 +17692,7 @@
         <f t="shared" si="10"/>
         <v>8.7119999999999997</v>
       </c>
-      <c r="F26" s="44">
-        <f>-'EB1'!I$7</f>
-        <v>194.51650000000001</v>
-      </c>
+      <c r="F26" s="44"/>
       <c r="H26" s="96"/>
       <c r="I26" s="96"/>
       <c r="J26" s="96" t="str">
@@ -17756,10 +17726,7 @@
         <f t="shared" si="10"/>
         <v>11.087999999999999</v>
       </c>
-      <c r="F27" s="44">
-        <f>-'EB1'!J$7</f>
-        <v>1500.6420000000001</v>
-      </c>
+      <c r="F27" s="44"/>
       <c r="H27" s="96"/>
       <c r="I27" s="96"/>
       <c r="J27" s="96" t="str">
@@ -17793,10 +17760,7 @@
         <f t="shared" si="10"/>
         <v>8.3160000000000007</v>
       </c>
-      <c r="F28" s="44">
-        <f>-'EB1'!K$7</f>
-        <v>400.84</v>
-      </c>
+      <c r="F28" s="44"/>
       <c r="H28" s="96"/>
       <c r="I28" s="96"/>
       <c r="J28" s="96" t="str">
@@ -17830,14 +17794,11 @@
         <f t="shared" si="10"/>
         <v>8.3160000000000007</v>
       </c>
-      <c r="F29" s="44">
-        <f>-'EB1'!L$7</f>
-        <v>1239.28</v>
-      </c>
+      <c r="F29" s="44"/>
       <c r="H29" s="96"/>
       <c r="I29" s="96"/>
       <c r="J29" s="96" t="str">
-        <f t="shared" si="8"/>
+        <f>$H$24&amp;C7&amp;1</f>
         <v>EXPHFO1</v>
       </c>
       <c r="K29" s="98" t="str">
@@ -17867,10 +17828,7 @@
         <f t="shared" si="10"/>
         <v>8.3160000000000007</v>
       </c>
-      <c r="F30" s="44">
-        <f>-'EB1'!M$7</f>
-        <v>453.036</v>
-      </c>
+      <c r="F30" s="44"/>
       <c r="H30" s="96"/>
       <c r="I30" s="96"/>
       <c r="J30" s="96" t="str">

</xml_diff>

<commit_message>
cHANGING IMPORT cost attribute from FLO_COST to COST
</commit_message>
<xml_diff>
--- a/VT_EE_UPS_V01.xlsx
+++ b/VT_EE_UPS_V01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEF09819-58BB-44AA-AC4E-A143ECD38405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B110F94D-8814-433C-A8F0-D3AFBF713ECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" tabRatio="901" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="901" firstSheet="1" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EB1" sheetId="133" r:id="rId1"/>
@@ -8153,7 +8153,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="181">
   <si>
     <t>CommName</t>
   </si>
@@ -8663,9 +8663,6 @@
   </si>
   <si>
     <t>NCAP_PASTI</t>
-  </si>
-  <si>
-    <t>FLO_COST</t>
   </si>
   <si>
     <t>NCAP_AF</t>
@@ -8719,6 +8716,8 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <charset val="186"/>
     </font>
     <font>
       <sz val="10"/>
@@ -13723,7 +13722,7 @@
         <v>6</v>
       </c>
       <c r="E12" s="53" t="s">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="F12" s="53" t="s">
         <v>169</v>
@@ -13732,7 +13731,7 @@
         <v>159</v>
       </c>
       <c r="H12" s="99" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="J12" s="93" t="s">
         <v>11</v>
@@ -14672,7 +14671,7 @@
   <sheetData>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D3" s="103">
         <v>2020</v>
@@ -14689,16 +14688,16 @@
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4" s="104" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B5" s="104"/>
       <c r="C5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D5">
         <v>369.77644024075659</v>
@@ -14716,7 +14715,7 @@
     <row r="6" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B6" s="104"/>
       <c r="C6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -15491,7 +15490,7 @@
       </c>
     </row>
     <row r="11" spans="2:26" x14ac:dyDescent="0.2">
-      <c r="B11" s="1" t="str">
+      <c r="B11" s="92" t="str">
         <f>K11</f>
         <v>MINSHL1</v>
       </c>
@@ -15788,7 +15787,7 @@
     </row>
     <row r="5" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C5">
         <v>3.5999999999999998E-6</v>
@@ -15848,16 +15847,16 @@
         <v>35</v>
       </c>
       <c r="G8" s="53" t="s">
+        <v>171</v>
+      </c>
+      <c r="H8" s="53" t="s">
         <v>172</v>
       </c>
-      <c r="H8" s="53" t="s">
+      <c r="I8" s="53" t="s">
         <v>173</v>
       </c>
-      <c r="I8" s="53" t="s">
+      <c r="J8" s="53" t="s">
         <v>174</v>
-      </c>
-      <c r="J8" s="53" t="s">
-        <v>175</v>
       </c>
       <c r="L8" s="93" t="s">
         <v>11</v>
@@ -15995,10 +15994,7 @@
         <f>$N$5</f>
         <v>GAS</v>
       </c>
-      <c r="F11" s="49">
-        <f>36/C5/1000000</f>
-        <v>10</v>
-      </c>
+      <c r="F11" s="49"/>
       <c r="G11" s="45">
         <f>'JRC-IDEES2023'!D5</f>
         <v>369.77644024075659</v>
@@ -16049,10 +16045,7 @@
         <f>$N$5</f>
         <v>GAS</v>
       </c>
-      <c r="F12" s="49">
-        <f>36/C5/1000000</f>
-        <v>10</v>
-      </c>
+      <c r="F12" s="49"/>
       <c r="G12" s="45"/>
       <c r="H12" s="45"/>
       <c r="I12" s="45"/>
@@ -17826,7 +17819,9 @@
         <f>J5</f>
         <v>MSW</v>
       </c>
-      <c r="E14" s="38"/>
+      <c r="E14" s="38">
+        <v>4.0500000000000007</v>
+      </c>
       <c r="F14" s="55"/>
       <c r="H14" s="92" t="str">
         <f>'EB1'!$B$5</f>

</xml_diff>